<commit_message>
chore: add history data-chart
</commit_message>
<xml_diff>
--- a/_08_api_invoke/背离统计-2026.xlsx
+++ b/_08_api_invoke/背离统计-2026.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="982" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="212">
   <si>
     <t>stock</t>
   </si>
@@ -601,9 +601,6 @@
   </si>
   <si>
     <t>wulf</t>
-  </si>
-  <si>
-    <t>clsk</t>
   </si>
   <si>
     <t>rklb</t>
@@ -1704,7 +1701,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:FI44"/>
+  <dimension ref="A1:FI43"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="125" max="165" width="9" style="2"/>
@@ -3941,124 +3938,145 @@
       </c>
     </row>
     <row r="26" spans="1:165">
-      <c r="A26" t="s">
-        <v>190</v>
-      </c>
-      <c r="D26" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="S26" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="Z26" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AD26" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AH26" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="AJ26" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="AL26" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AM26" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="AN26" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AP26" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AS26" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="AU26" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="BC26" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="BM26" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="BS26" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="BT26" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="BW26" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="CE26" s="6" t="s">
-        <v>163</v>
-      </c>
       <c r="CM26" s="1"/>
-      <c r="CO26" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="CU26" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="DA26" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="DQ26" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="DT26" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="EH26" s="11" t="s">
-        <v>163</v>
-      </c>
     </row>
     <row r="27" spans="1:165">
       <c r="CM27" s="1"/>
     </row>
     <row r="28" spans="1:165">
+      <c r="A28" t="s">
+        <v>190</v>
+      </c>
+      <c r="R28" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="Y28" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="AJ28" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="AN28" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="AP28" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="AS28" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="AU28" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="BD28" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="BN28" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="BU28" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="BW28" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="CF28" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="CH28" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="CJ28" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="CK28" s="6" t="s">
+        <v>163</v>
+      </c>
       <c r="CM28" s="1"/>
+      <c r="CO28" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="CQ28" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="CV28" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="CW28" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="CY28" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="DB28" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="DC28" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="DF28" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="DM28" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="DY28" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="EH28" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="EZ28" s="9" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="29" spans="1:165">
       <c r="A29" t="s">
         <v>191</v>
       </c>
+      <c r="H29" s="6" t="s">
+        <v>163</v>
+      </c>
       <c r="R29" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="Y29" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="AJ29" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="AN29" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="AP29" s="6" t="s">
+      <c r="X29" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="AG29" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="AH29" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="AM29" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="AN29" s="6" t="s">
         <v>162</v>
       </c>
       <c r="AS29" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="AU29" s="8" t="s">
-        <v>165</v>
+      <c r="AT29" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="AV29" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="BC29" s="7" t="s">
+        <v>166</v>
       </c>
       <c r="BD29" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="BN29" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="BU29" s="7" t="s">
+      <c r="BK29" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="BR29" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="BT29" s="7" t="s">
         <v>166</v>
       </c>
       <c r="BW29" s="7" t="s">
@@ -4067,50 +4085,38 @@
       <c r="CF29" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="CH29" s="6" t="s">
-        <v>162</v>
-      </c>
       <c r="CJ29" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="CK29" s="6" t="s">
         <v>163</v>
       </c>
       <c r="CM29" s="1"/>
-      <c r="CO29" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="CQ29" s="6" t="s">
-        <v>162</v>
+      <c r="CO29" s="7" t="s">
+        <v>164</v>
       </c>
       <c r="CV29" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="CW29" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="CY29" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="DB29" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="DC29" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="DF29" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="DM29" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="DY29" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="EH29" s="11" t="s">
-        <v>163</v>
-      </c>
-      <c r="EZ29" s="9" t="s">
+      <c r="CX29" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="DE29" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="DG29" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="DI29" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="DM29" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="DZ29" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="ED29" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="ES29" s="9" t="s">
         <v>164</v>
       </c>
     </row>
@@ -4118,792 +4124,702 @@
       <c r="A30" t="s">
         <v>192</v>
       </c>
-      <c r="H30" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="R30" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="X30" s="7" t="s">
+      <c r="B30" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="K30" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="M30" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="Q30" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="U30" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="X30" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="AC30" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="AF30" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="AM30" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="AO30" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="AR30" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="BB30" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="AG30" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AH30" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="AM30" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="AN30" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AS30" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="AT30" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="AV30" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="BC30" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="BD30" s="7" t="s">
-        <v>164</v>
+      <c r="BH30" s="7" t="s">
+        <v>166</v>
       </c>
       <c r="BK30" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="BR30" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="BT30" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="BW30" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="CF30" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="CJ30" s="6" t="s">
-        <v>163</v>
+      <c r="BL30" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="BV30" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="BY30" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="CE30" s="6" t="s">
+        <v>162</v>
       </c>
       <c r="CM30" s="1"/>
       <c r="CO30" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="CV30" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="CX30" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="DE30" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="DG30" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="DI30" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="DM30" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="DZ30" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="ED30" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="ES30" s="9" t="s">
+      <c r="CW30" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="CX30" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="CY30" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="DL30" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="DP30" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="EC30" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="FC30" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="FD30" s="9" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="31" spans="1:165">
-      <c r="A31" t="s">
-        <v>193</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="K31" s="8" t="s">
-        <v>174</v>
-      </c>
-      <c r="M31" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="Q31" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="U31" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="X31" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="AC31" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="AF31" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AM31" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="AO31" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AR31" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="BB31" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="BH31" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="BK31" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="BL31" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="BV31" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="BY31" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="CE31" s="6" t="s">
-        <v>162</v>
-      </c>
       <c r="CM31" s="1"/>
-      <c r="CO31" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="CW31" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="CX31" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="CY31" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="DL31" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="DP31" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="EC31" s="11" t="s">
-        <v>163</v>
-      </c>
-      <c r="FC31" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="FD31" s="9" t="s">
-        <v>164</v>
-      </c>
     </row>
     <row r="32" spans="1:165">
       <c r="CM32" s="1"/>
     </row>
     <row r="33" spans="1:165">
+      <c r="A33" t="s">
+        <v>193</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="K33" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="M33" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="P33" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="W33" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="Z33" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="AC33" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="AF33" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="AK33" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="AL33" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="AM33" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="AT33" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="AV33" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="BC33" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="BF33" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="BI33" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="BJ33" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="BU33" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="BW33" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="CF33" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="CG33" s="6" t="s">
+        <v>163</v>
+      </c>
       <c r="CM33" s="1"/>
+      <c r="CN33" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="CO33" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="DC33" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="DD33" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="DF33" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="DH33" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="DL33" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="DM33" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="DQ33" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="EF33" s="10" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="34" spans="1:165">
       <c r="A34" t="s">
         <v>194</v>
       </c>
-      <c r="C34" s="8" t="s">
-        <v>174</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="H34" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="K34" s="8" t="s">
-        <v>165</v>
+      <c r="I34" s="6" t="s">
+        <v>163</v>
       </c>
       <c r="M34" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="P34" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="W34" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="Z34" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AC34" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AF34" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="AK34" s="7" t="s">
-        <v>164</v>
+      <c r="R34" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="AC34" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="AJ34" s="8" t="s">
+        <v>165</v>
       </c>
       <c r="AL34" s="8" t="s">
         <v>165</v>
       </c>
-      <c r="AM34" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AT34" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="AV34" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="BC34" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="BF34" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="BI34" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="BJ34" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="BU34" s="7" t="s">
+      <c r="AP34" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="AT34" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="AU34" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="AW34" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="BH34" s="7" t="s">
         <v>164</v>
       </c>
       <c r="BW34" s="7" t="s">
         <v>166</v>
       </c>
+      <c r="BX34" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="CC34" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="CE34" s="8" t="s">
+        <v>165</v>
+      </c>
       <c r="CF34" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="CG34" s="6" t="s">
+      <c r="CH34" s="6" t="s">
         <v>163</v>
       </c>
       <c r="CM34" s="1"/>
       <c r="CN34" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="CO34" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="DC34" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="DD34" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="DF34" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="DH34" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="DL34" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="DM34" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="DQ34" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="EF34" s="10" t="s">
-        <v>165</v>
+        <v>164</v>
+      </c>
+      <c r="CP34" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="CQ34" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="CV34" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="DC34" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="DG34" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="DI34" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="DZ34" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="ED34" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="EH34" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="FC34" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="FE34" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="FH34" s="9" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="35" spans="1:165">
       <c r="A35" t="s">
         <v>195</v>
       </c>
-      <c r="I35" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="M35" s="6" t="s">
-        <v>162</v>
+      <c r="J35" s="7" t="s">
+        <v>164</v>
       </c>
       <c r="R35" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AC35" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="AJ35" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="AL35" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="AP35" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AT35" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="AU35" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="AW35" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="BH35" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="BW35" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="BX35" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="CC35" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="CE35" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="CF35" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
+      </c>
+      <c r="AB35" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="AG35" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="AM35" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="AS35" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="BC35" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="BK35" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="BT35" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="BV35" s="6" t="s">
+        <v>163</v>
       </c>
       <c r="CH35" s="6" t="s">
         <v>163</v>
       </c>
+      <c r="CL35" s="7" t="s">
+        <v>166</v>
+      </c>
       <c r="CM35" s="1"/>
-      <c r="CN35" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="CP35" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="CQ35" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="CV35" s="8" t="s">
-        <v>174</v>
-      </c>
-      <c r="DC35" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="DG35" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="DI35" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="DZ35" s="9" t="s">
-        <v>178</v>
-      </c>
-      <c r="ED35" s="9" t="s">
+      <c r="CO35" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="CU35" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="CY35" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="DC35" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="DL35" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="DM35" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="DQ35" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="DT35" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="DY35" s="9" t="s">
         <v>166</v>
       </c>
       <c r="EH35" s="11" t="s">
         <v>163</v>
       </c>
+      <c r="EW35" s="9" t="s">
+        <v>166</v>
+      </c>
       <c r="FC35" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="FE35" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="FH35" s="9" t="s">
-        <v>178</v>
+      <c r="FG35" s="9" t="s">
+        <v>166</v>
       </c>
     </row>
-    <row r="36" spans="1:165">
+    <row r="36" customFormat="1" spans="1:165">
       <c r="A36" t="s">
         <v>196</v>
       </c>
-      <c r="J36" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="R36" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="AB36" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AG36" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="AM36" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="AS36" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="BC36" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="BK36" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="BT36" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="BV36" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="CH36" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="CL36" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="CM36" s="1"/>
-      <c r="CO36" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="CU36" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="CY36" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="DC36" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="DL36" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="DM36" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="DQ36" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="DT36" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="DY36" s="9" t="s">
-        <v>166</v>
-      </c>
+      <c r="DM36" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="EG36" s="2"/>
       <c r="EH36" s="11" t="s">
         <v>163</v>
       </c>
-      <c r="EW36" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="FC36" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="FG36" s="9" t="s">
-        <v>166</v>
-      </c>
+      <c r="EI36" s="2"/>
+      <c r="EJ36" s="2"/>
+      <c r="EK36" s="2"/>
+      <c r="EL36" s="2"/>
+      <c r="EM36" s="2"/>
+      <c r="EN36" s="2"/>
+      <c r="EO36" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="EP36" s="2"/>
+      <c r="EQ36" s="2"/>
+      <c r="ER36" s="2"/>
+      <c r="ES36" s="2"/>
+      <c r="ET36" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="EU36" s="2"/>
+      <c r="EV36" s="2"/>
+      <c r="EW36" s="2"/>
+      <c r="EX36" s="2"/>
+      <c r="EY36" s="2"/>
+      <c r="EZ36" s="2"/>
+      <c r="FA36" s="2"/>
+      <c r="FB36" s="2"/>
+      <c r="FC36" s="2"/>
+      <c r="FD36" s="2"/>
+      <c r="FE36" s="2"/>
+      <c r="FF36" s="2"/>
+      <c r="FG36" s="2"/>
+      <c r="FH36" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="FI36" s="2"/>
     </row>
-    <row r="37" customFormat="1" spans="1:165">
-      <c r="A37" t="s">
-        <v>197</v>
-      </c>
-      <c r="DM37" s="10" t="s">
-        <v>165</v>
-      </c>
-      <c r="EG37" s="2"/>
-      <c r="EH37" s="11" t="s">
-        <v>163</v>
-      </c>
-      <c r="EI37" s="2"/>
-      <c r="EJ37" s="2"/>
-      <c r="EK37" s="2"/>
-      <c r="EL37" s="2"/>
-      <c r="EM37" s="2"/>
-      <c r="EN37" s="2"/>
-      <c r="EO37" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="EP37" s="2"/>
-      <c r="EQ37" s="2"/>
-      <c r="ER37" s="2"/>
-      <c r="ES37" s="2"/>
-      <c r="ET37" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="EU37" s="2"/>
-      <c r="EV37" s="2"/>
-      <c r="EW37" s="2"/>
-      <c r="EX37" s="2"/>
-      <c r="EY37" s="2"/>
-      <c r="EZ37" s="2"/>
-      <c r="FA37" s="2"/>
-      <c r="FB37" s="2"/>
-      <c r="FC37" s="2"/>
-      <c r="FD37" s="2"/>
-      <c r="FE37" s="2"/>
-      <c r="FF37" s="2"/>
-      <c r="FG37" s="2"/>
-      <c r="FH37" s="11" t="s">
-        <v>163</v>
-      </c>
-      <c r="FI37" s="2"/>
+    <row r="37" spans="1:165">
+      <c r="CM37" s="1"/>
     </row>
     <row r="38" spans="1:165">
       <c r="CM38" s="1"/>
     </row>
     <row r="39" spans="1:165">
+      <c r="A39" t="s">
+        <v>197</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="G39" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="U39" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="Y39" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="AF39" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="AG39" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="AL39" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="AM39" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="AO39" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="AQ39" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="AY39" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="BG39" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="BU39" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="BW39" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="CE39" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="CG39" s="6" t="s">
+        <v>162</v>
+      </c>
       <c r="CM39" s="1"/>
+      <c r="CO39" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="DG39" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="DI39" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="DJ39" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="DN39" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="DQ39" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="DT39" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="DY39" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="ET39" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="EX39" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="EZ39" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="FC39" s="9" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="40" spans="1:165">
       <c r="A40" t="s">
         <v>198</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="G40" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="U40" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="Y40" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="AF40" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="M40" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="AA40" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="AB40" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="AE40" s="6" t="s">
         <v>162</v>
       </c>
       <c r="AG40" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="AL40" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AM40" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="AO40" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="AQ40" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="AY40" s="7" t="s">
-        <v>164</v>
+        <v>162</v>
+      </c>
+      <c r="AL40" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="BD40" s="8" t="s">
+        <v>165</v>
       </c>
       <c r="BG40" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="BU40" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="BH40" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="BJ40" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="BS40" s="7" t="s">
         <v>166</v>
       </c>
       <c r="BW40" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="CE40" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="CG40" s="6" t="s">
-        <v>162</v>
+      <c r="BX40" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="CF40" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="CI40" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="CJ40" s="6" t="s">
+        <v>163</v>
       </c>
       <c r="CM40" s="1"/>
       <c r="CO40" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="DG40" s="7" t="s">
-        <v>166</v>
+      <c r="CP40" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="CX40" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="DF40" s="6" t="s">
+        <v>163</v>
       </c>
       <c r="DI40" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="DJ40" s="7" t="s">
-        <v>164</v>
-      </c>
       <c r="DN40" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="DQ40" s="7" t="s">
-        <v>166</v>
-      </c>
       <c r="DT40" s="7" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="DY40" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="ET40" s="9" t="s">
-        <v>164</v>
+      <c r="EL40" s="11" t="s">
+        <v>162</v>
       </c>
       <c r="EX40" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="EZ40" s="9" t="s">
         <v>164</v>
       </c>
       <c r="FC40" s="9" t="s">
         <v>166</v>
       </c>
+      <c r="FD40" s="9" t="s">
+        <v>164</v>
+      </c>
     </row>
-    <row r="41" spans="1:165">
-      <c r="A41" t="s">
+    <row r="42" spans="1:165">
+      <c r="AO42" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="B41" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="D41" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="M41" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="AA41" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AB41" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="AE41" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AG41" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="AL41" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="BD41" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="BG41" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="BH41" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="BJ41" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="BS41" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="BW41" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="BX41" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="CF41" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="CI41" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="CJ41" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="CM41" s="1"/>
-      <c r="CO41" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="CP41" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="CX41" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="DF41" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="DI41" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="DN41" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="DT41" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="DY41" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="EL41" s="11" t="s">
-        <v>162</v>
-      </c>
-      <c r="EX41" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="FC41" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="FD41" s="9" t="s">
-        <v>164</v>
+      <c r="BF42" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="BN42" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="BV42" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="BW42" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="BX42" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="CH42" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="CM42" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="CN42" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="CO42" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="DN42" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="DQ42" t="s">
+        <v>209</v>
+      </c>
+      <c r="EH42" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="FC42" s="2" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="43" spans="1:165">
-      <c r="AO43" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="BF43" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="BN43" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="BV43" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="BW43" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="BX43" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="CH43" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="CM43" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="CN43" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="CO43" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="DN43" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="DQ43" t="s">
-        <v>210</v>
-      </c>
-      <c r="EH43" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="FC43" s="2" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="44" spans="1:165">
-      <c r="BV44">
+      <c r="BV43">
         <v>-2.37</v>
       </c>
-      <c r="CJ44">
+      <c r="CJ43">
         <v>-1.91</v>
       </c>
-      <c r="CK44">
+      <c r="CK43">
         <v>-0.5</v>
       </c>
-      <c r="CL44">
+      <c r="CL43">
         <v>0.2</v>
       </c>
-      <c r="CM44">
+      <c r="CM43">
         <v>-1.85</v>
       </c>
-      <c r="CN44">
+      <c r="CN43">
         <v>1.45</v>
       </c>
-      <c r="CO44">
+      <c r="CO43">
         <v>1.3</v>
       </c>
-      <c r="DQ44">
+      <c r="DQ43">
         <v>-1.54</v>
       </c>
-      <c r="DR44">
+      <c r="DR43">
         <v>-1.75</v>
       </c>
-      <c r="DS44">
+      <c r="DS43">
         <v>-1.44</v>
       </c>
-      <c r="FA44" s="2">
+      <c r="FA43" s="2">
         <v>-2.39</v>
       </c>
-      <c r="FB44" s="2">
+      <c r="FB43" s="2">
         <v>-1.95</v>
       </c>
-      <c r="FC44" s="2">
+      <c r="FC43" s="2">
         <v>-0.76</v>
       </c>
-      <c r="FD44" s="2">
+      <c r="FD43" s="2">
         <v>3.39</v>
       </c>
     </row>

</xml_diff>